<commit_message>
Backfill weekly dashboard history for 2026-09-14 through 2026-09-20.
Use the new planner sales export and refresh daily summary pages with the latest business date.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/每日输出/小短/郑州-小短-风灵个微全天在线率&爱芯后台授权.xlsx
+++ b/每日输出/小短/郑州-小短-风灵个微全天在线率&爱芯后台授权.xlsx
@@ -21,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -49,8 +49,19 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <color rgb="0000B050"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <b val="1"/>
       <color rgb="00C00000"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="0000B050"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -201,22 +212,22 @@
     <xf numFmtId="10" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="9" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="9" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="9" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="9" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="9" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="9" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -584,13 +595,1300 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:R15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>无数据</t>
+          <t>服务期</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>日期</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>学段</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>分部</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>阶段</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>运营中心</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>战队</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>学习规划师</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>学习规划师姓名</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>带班产品</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>风灵微信在线率</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>不在线时段list</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>年级</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>学部</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>辅导老师</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>辅导姓名</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>sys_source</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>分组</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>20260918</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>爱学</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>短期班</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>全部</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>郑州</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>仵夏炎</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>peifang</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>裴芳</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>低价课</t>
+        </is>
+      </c>
+      <c r="K2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>6,7,8,9,10,11,12,13,14,15,16,17,18,19,20,21,22,23</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>全年级</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>小学</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>peifang</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>裴芳</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>爱学</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>小短</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>20260918</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>爱学</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>短期班</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>全部</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>郑州</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>秦淑楠</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>lijingzhe</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>李京哲</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>低价课</t>
+        </is>
+      </c>
+      <c r="K3" t="n">
+        <v>1</v>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>全年级</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>小学</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>lijingzhe</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>李京哲</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>爱学</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>小短</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>20260918</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>爱学</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>短期班</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>全部</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>郑州</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>秦淑楠</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>wangmengdi01</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>王梦迪</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>低价课</t>
+        </is>
+      </c>
+      <c r="K4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>6,7,8,9,10,11,12,13,14,15,16,17,18,19,20,21,22,23</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>全年级</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>小学</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>wangmengdi01</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>王梦迪</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>爱学</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>小短</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>20260918</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>爱学</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>短期班</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>全部</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>郑州</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>秦淑楠</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>lishaohui</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>李少辉</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>低价课</t>
+        </is>
+      </c>
+      <c r="K5" t="n">
+        <v>1</v>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>全年级</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>小学</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>lishaohui</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>李少辉</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>爱学</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>小短</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>20260918</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>爱学</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>短期班</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>全部</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>郑州</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>仵夏炎</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>chenxiangru</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>陈湘茹</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>低价课</t>
+        </is>
+      </c>
+      <c r="K6" t="n">
+        <v>1</v>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>全年级</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>小学</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>chenxiangru</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>陈湘茹</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>爱学</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>小短</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>20260918</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>爱学</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>短期班</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>全部</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>郑州</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>秦淑楠</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>wangcongyang</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>王聪阳</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>低价课</t>
+        </is>
+      </c>
+      <c r="K7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>6,7,8,9,10,11,12,13,14,15,16,17,18,19,20,21,22,23</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>全年级</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>小学</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>wangcongyang</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>王聪阳</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>爱学</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>小短</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>20260918</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>爱学</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>短期班</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>全部</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>郑州</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>仵夏炎</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>wangxinran</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>王欣冉</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>低价课</t>
+        </is>
+      </c>
+      <c r="K8" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>6,7,8,9,10,11,12,13,14,15,16,17,18,19,20,21,22,23</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>全年级</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>小学</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>wangxinran</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>王欣冉</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>爱学</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>小短</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>20260918</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>爱学</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>短期班</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>全部</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>郑州</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>秦淑楠</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>yangxiju</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>杨喜菊</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>低价课</t>
+        </is>
+      </c>
+      <c r="K9" t="n">
+        <v>1</v>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>全年级</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>小学</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>yangxiju</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>杨喜菊</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>爱学</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>小短</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>20260918</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>爱学</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>短期班</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>全部</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>郑州</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>仵夏炎</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>jingyabo</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>荆雅博</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>低价课</t>
+        </is>
+      </c>
+      <c r="K10" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>6,7,8,9,10,11,12,13,14,15,16,17,18,19,20,21,22,23</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>全年级</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>小学</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>jingyabo</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>荆雅博</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>爱学</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>小短</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>20260918</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>爱学</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>短期班</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>全部</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>郑州</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>仵夏炎</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>liudonghui</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>刘栋辉</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>低价课</t>
+        </is>
+      </c>
+      <c r="K11" t="n">
+        <v>0</v>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>6,7,8,9,10,11,12,13,14,15,16,17,18,19,20,21,22,23</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>全年级</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>小学</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>liudonghui</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>刘栋辉</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>爱学</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>小短</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>20260918</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>爱学</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>短期班</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>全部</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>郑州</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>仵夏炎</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>lvzhiheng</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>吕志恒</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>低价课</t>
+        </is>
+      </c>
+      <c r="K12" t="n">
+        <v>1</v>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>全年级</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>小学</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>lvzhiheng</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>吕志恒</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>爱学</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>小短</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>20260918</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>爱学</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>短期班</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>全部</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>郑州</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>仵夏炎</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>wuxiayan</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>仵夏炎</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>低价课</t>
+        </is>
+      </c>
+      <c r="K13" t="n">
+        <v>0</v>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>6,7,8,9,10,11,12,13,14,15,16,17,18,19,20,21,22,23</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>全年级</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>小学</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>wuxiayan</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>仵夏炎</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>爱学</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>小短</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>20260918</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>爱学</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>短期班</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>全部</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>郑州</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>秦淑楠</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>zhangyuying01</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>张昱莹</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>低价课</t>
+        </is>
+      </c>
+      <c r="K14" t="n">
+        <v>0</v>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>6,7,8,9,10,11,12,13,14,15,16,17,18,19,20,21,22,23</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>全年级</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>小学</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>zhangyuying01</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>张昱莹</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>爱学</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>小短</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>20260918</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>爱学</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>短期班</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>全部</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>郑州</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>秦淑楠</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>lidanyang</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>李丹阳</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>低价课</t>
+        </is>
+      </c>
+      <c r="K15" t="n">
+        <v>1</v>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>全年级</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>小学</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>lidanyang</t>
+        </is>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>李丹阳</t>
+        </is>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>爱学</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>小短</t>
         </is>
       </c>
     </row>
@@ -605,14 +1903,91 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>无数据</t>
-        </is>
+          <t>学部</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>年级</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>战队</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>低价课带班</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>全天在线</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>个微全天在线率</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>小学</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>全年级</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>仵夏炎</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>7</v>
+      </c>
+      <c r="E2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0.2857142857142857</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>小学</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>全年级</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>秦淑楠</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>7</v>
+      </c>
+      <c r="E3" t="n">
+        <v>4</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.5714285714285714</v>
       </c>
     </row>
   </sheetData>
@@ -645,7 +2020,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>个微-风灵全天在线率及爱芯授权功能正常率（小短） 9月6日</t>
+          <t>个微-风灵全天在线率及爱芯授权功能正常率（小短） 9月20日</t>
         </is>
       </c>
       <c r="B1" s="7" t="n"/>
@@ -733,28 +2108,28 @@
         </is>
       </c>
       <c r="D3" s="3" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F3" s="8" t="n">
-        <v>0</v>
+        <v>0.2857142857142857</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="H3" s="3" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="I3" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="J3" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="K3" s="9" t="e">
-        <v>#N/A</v>
+        <v>2</v>
+      </c>
+      <c r="J3" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="K3" s="8" t="n">
+        <v>0.2857142857142857</v>
       </c>
     </row>
     <row r="4">
@@ -766,28 +2141,28 @@
         </is>
       </c>
       <c r="D4" s="3" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F4" s="8" t="n">
-        <v>0</v>
+        <v>0.5714285714285714</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="I4" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="J4" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="K4" s="9" t="e">
-        <v>#N/A</v>
+        <v>4</v>
+      </c>
+      <c r="J4" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="K4" s="8" t="n">
+        <v>0.5714285714285714</v>
       </c>
     </row>
     <row r="5">
@@ -799,28 +2174,28 @@
       </c>
       <c r="C5" s="10" t="n"/>
       <c r="D5" s="10" t="n">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="E5" s="10" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="F5" s="11" t="n">
-        <v>0</v>
+        <v>0.4285714285714285</v>
       </c>
       <c r="G5" s="10" t="n">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="H5" s="10" t="n">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="I5" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="J5" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="K5" s="12" t="e">
-        <v>#N/A</v>
+        <v>6</v>
+      </c>
+      <c r="J5" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="K5" s="11" t="n">
+        <v>0.4285714285714285</v>
       </c>
     </row>
     <row r="6">
@@ -836,28 +2211,28 @@
       </c>
       <c r="C6" s="10" t="inlineStr"/>
       <c r="D6" s="10" t="n">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="E6" s="10" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="F6" s="11" t="n">
-        <v>0</v>
+        <v>0.4285714285714285</v>
       </c>
       <c r="G6" s="10" t="n">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="H6" s="10" t="n">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="I6" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="J6" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="K6" s="12" t="e">
-        <v>#N/A</v>
+        <v>6</v>
+      </c>
+      <c r="J6" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="K6" s="11" t="n">
+        <v>0.4285714285714285</v>
       </c>
     </row>
   </sheetData>
@@ -904,14 +2279,778 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:K15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>无数据</t>
-        </is>
+          <t>日期</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>分组</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>学部</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>年级</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>战队</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>老师邮箱</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>老师姓名</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>个微授权</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>整体正常</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>运营中心</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>小时</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>小短</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>小学</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>全年级</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>仵夏炎</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>chenxiangru</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>陈湘茹</t>
+        </is>
+      </c>
+      <c r="H2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>郑州</t>
+        </is>
+      </c>
+      <c r="K2" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>小短</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>小学</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>全年级</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>仵夏炎</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>jingyabo</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>荆雅博</t>
+        </is>
+      </c>
+      <c r="H3" t="n">
+        <v>1</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>郑州</t>
+        </is>
+      </c>
+      <c r="K3" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>小短</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>小学</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>全年级</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>仵夏炎</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>liudonghui</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>刘栋辉</t>
+        </is>
+      </c>
+      <c r="H4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>郑州</t>
+        </is>
+      </c>
+      <c r="K4" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>小短</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>小学</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>全年级</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>仵夏炎</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>lvzhiheng</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>吕志恒</t>
+        </is>
+      </c>
+      <c r="H5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I5" t="n">
+        <v>1</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>郑州</t>
+        </is>
+      </c>
+      <c r="K5" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>小短</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>小学</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>全年级</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>仵夏炎</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>peifang</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>裴芳</t>
+        </is>
+      </c>
+      <c r="H6" t="n">
+        <v>1</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>郑州</t>
+        </is>
+      </c>
+      <c r="K6" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>小短</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>小学</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>全年级</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>仵夏炎</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>wangxinran</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>王欣冉</t>
+        </is>
+      </c>
+      <c r="H7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>郑州</t>
+        </is>
+      </c>
+      <c r="K7" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>小短</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>小学</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>全年级</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>仵夏炎</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>wuxiayan</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>仵夏炎</t>
+        </is>
+      </c>
+      <c r="H8" t="n">
+        <v>1</v>
+      </c>
+      <c r="I8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>郑州</t>
+        </is>
+      </c>
+      <c r="K8" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>小短</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>小学</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>全年级</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>秦淑楠</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>lidanyang</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>李丹阳</t>
+        </is>
+      </c>
+      <c r="H9" t="n">
+        <v>1</v>
+      </c>
+      <c r="I9" t="n">
+        <v>1</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>郑州</t>
+        </is>
+      </c>
+      <c r="K9" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>小短</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>小学</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>全年级</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>秦淑楠</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>lijingzhe</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>李京哲</t>
+        </is>
+      </c>
+      <c r="H10" t="n">
+        <v>1</v>
+      </c>
+      <c r="I10" t="n">
+        <v>1</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>郑州</t>
+        </is>
+      </c>
+      <c r="K10" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>小短</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>小学</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>全年级</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>秦淑楠</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>lishaohui</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>李少辉</t>
+        </is>
+      </c>
+      <c r="H11" t="n">
+        <v>1</v>
+      </c>
+      <c r="I11" t="n">
+        <v>1</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>郑州</t>
+        </is>
+      </c>
+      <c r="K11" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>小短</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>小学</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>全年级</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>秦淑楠</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>wangcongyang</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>王聪阳</t>
+        </is>
+      </c>
+      <c r="H12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I12" t="n">
+        <v>0</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>郑州</t>
+        </is>
+      </c>
+      <c r="K12" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>小短</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>小学</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>全年级</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>秦淑楠</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>wangmengdi01</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>王梦迪</t>
+        </is>
+      </c>
+      <c r="H13" t="n">
+        <v>1</v>
+      </c>
+      <c r="I13" t="n">
+        <v>0</v>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>郑州</t>
+        </is>
+      </c>
+      <c r="K13" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>小短</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>小学</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>全年级</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>秦淑楠</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>yangxiju</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>杨喜菊</t>
+        </is>
+      </c>
+      <c r="H14" t="n">
+        <v>1</v>
+      </c>
+      <c r="I14" t="n">
+        <v>1</v>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>郑州</t>
+        </is>
+      </c>
+      <c r="K14" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>小短</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>小学</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>全年级</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>秦淑楠</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>zhangyuying01</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>张昱莹</t>
+        </is>
+      </c>
+      <c r="H15" t="n">
+        <v>1</v>
+      </c>
+      <c r="I15" t="n">
+        <v>0</v>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>郑州</t>
+        </is>
+      </c>
+      <c r="K15" t="n">
+        <v>22</v>
       </c>
     </row>
   </sheetData>
@@ -987,16 +3126,19 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="E2" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="F2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G2" t="n">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0.2857142857142857</v>
       </c>
     </row>
     <row r="3">
@@ -1016,16 +3158,19 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="E3" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="F3" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G3" t="n">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0.5714285714285714</v>
       </c>
     </row>
   </sheetData>

</xml_diff>